<commit_message>
Add orbiting resource enemy wave
</commit_message>
<xml_diff>
--- a/Luban/Datas/Wave.xlsx
+++ b/Luban/Datas/Wave.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="12.33203125" customWidth="1" style="1" min="1" max="2"/>
@@ -817,219 +817,237 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_01</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>level_01</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_02</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>level_02</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_03</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>level_03</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_04</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>level_04</t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_05</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>level_05</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_06</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>level_06</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_07</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>level_07</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_08</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>level_08</t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_09</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>level_09</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_10</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>level_10</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_11</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>level_11</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="0" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>wave_boss_final_12</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>level_12</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>180</v>
+      <c r="E28" s="0" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>26</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>wave_level_01_resource_orbit</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>level_01</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add three resource enemy flight waves
</commit_message>
<xml_diff>
--- a/Luban/Datas/Wave.xlsx
+++ b/Luban/Datas/Wave.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="12.33203125" customWidth="1" style="1" min="1" max="2"/>
@@ -1033,21 +1033,75 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>wave_level_01_resource_orbit</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>level_01</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="0" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="n">
+        <v>27</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>wave_level_01_resource_left_downright</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>level_01</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>28</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>wave_level_01_resource_right_downleft</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>level_01</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>29</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>wave_level_01_resource_top_down</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>level_01</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>